<commit_message>
Nang cap nhap sinh vien theo ma lop va xem truoc Excel
</commit_message>
<xml_diff>
--- a/backend/nhap_excel/mau_excel/mau_nhap_sinh_vien_theo_lop.xlsx
+++ b/backend/nhap_excel/mau_excel/mau_nhap_sinh_vien_theo_lop.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dữ liệu" sheetId="1" r:id="Rbeff2835bc4d41f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ví dụ" sheetId="2" r:id="R97a78878d64d4e90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="3" r:id="R09d68d2986164d30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh mục" sheetId="4" r:id="Rb0debb37332e4e8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hệ thống" sheetId="5" r:id="R3a0704097060418a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dữ liệu" sheetId="1" r:id="Ra1d41e9770f94e72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ví dụ" sheetId="2" r:id="R56ead8fef4d94542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="3" r:id="R5354a65722f04285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh mục" sheetId="4" r:id="R1e44d13ba23040f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hệ thống" sheetId="5" r:id="R332f7a4dcb914749"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -56,7 +56,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -113,8 +113,13 @@
         <x:fgColor rgb="FFF4B183"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF5B9BD5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="30">
+  <x:borders count="31">
     <x:border/>
     <x:border/>
     <x:border>
@@ -341,11 +346,25 @@
         <x:color rgb="FFAAB7B8"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF7F8C8D"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF7F8C8D"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF7F8C8D"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF7F8C8D"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="230">
+  <x:cellXfs count="236">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -872,6 +891,18 @@
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1039,6 +1070,7 @@
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -1048,10 +1080,10 @@
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="13" t="str">
-        <x:v>Nhập dữ liệu từ dòng 4 trở xuống. Không đổi tên/không đổi thứ tự cột. Mã khoa và Khóa học được tự động lấy từ lớp; tài khoản mặc định Đang hoạt động.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="34" customHeight="1">
+        <x:v>Nhập dữ liệu từ dòng 4 trở xuống. Không đổi tên/không đổi thứ tự cột. Mỗi sinh viên phải có Mã lớp; hệ thống tự lấy Khoa và Khóa học từ lớp trùng mã.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="29" t="str">
         <x:v>STT</x:v>
       </x:c>
@@ -1068,21 +1100,24 @@
         <x:v>Mật khẩu</x:v>
       </x:c>
       <x:c r="F3" s="30" t="str">
+        <x:v>Mã lớp</x:v>
+      </x:c>
+      <x:c r="G3" s="30" t="str">
         <x:v>Ngày sinh</x:v>
       </x:c>
-      <x:c r="G3" s="30" t="str">
+      <x:c r="H3" s="30" t="str">
         <x:v>Giới tính</x:v>
       </x:c>
-      <x:c r="H3" s="30" t="str">
+      <x:c r="I3" s="30" t="str">
         <x:v>Số điện thoại</x:v>
       </x:c>
-      <x:c r="I3" s="30" t="str">
+      <x:c r="J3" s="30" t="str">
         <x:v>CCCD</x:v>
       </x:c>
-      <x:c r="J3" s="30" t="str">
+      <x:c r="K3" s="31" t="str">
         <x:v>Địa chỉ</x:v>
       </x:c>
-      <x:c r="K3" s="31" t="str">
+      <x:c r="L3" s="235" t="str">
         <x:v>Trạng thái sinh viên</x:v>
       </x:c>
     </x:row>
@@ -1100,6 +1135,7 @@
       <x:c r="I4" s="127"/>
       <x:c r="J4" s="100"/>
       <x:c r="K4" s="101"/>
+      <x:c r="L4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="112" t="n">
@@ -1115,6 +1151,7 @@
       <x:c r="I5" s="128"/>
       <x:c r="J5" s="68"/>
       <x:c r="K5" s="69"/>
+      <x:c r="L5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="113" t="n">
@@ -1130,6 +1167,7 @@
       <x:c r="I6" s="129"/>
       <x:c r="J6" s="106"/>
       <x:c r="K6" s="107"/>
+      <x:c r="L6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="112" t="n">
@@ -1145,6 +1183,7 @@
       <x:c r="I7" s="128"/>
       <x:c r="J7" s="68"/>
       <x:c r="K7" s="69"/>
+      <x:c r="L7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="113" t="n">
@@ -1160,6 +1199,7 @@
       <x:c r="I8" s="129"/>
       <x:c r="J8" s="106"/>
       <x:c r="K8" s="107"/>
+      <x:c r="L8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="112" t="n">
@@ -1175,6 +1215,7 @@
       <x:c r="I9" s="128"/>
       <x:c r="J9" s="68"/>
       <x:c r="K9" s="69"/>
+      <x:c r="L9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="113" t="n">
@@ -1190,6 +1231,7 @@
       <x:c r="I10" s="129"/>
       <x:c r="J10" s="106"/>
       <x:c r="K10" s="107"/>
+      <x:c r="L10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="112" t="n">
@@ -1205,6 +1247,7 @@
       <x:c r="I11" s="128"/>
       <x:c r="J11" s="68"/>
       <x:c r="K11" s="69"/>
+      <x:c r="L11"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="113" t="n">
@@ -1220,6 +1263,7 @@
       <x:c r="I12" s="129"/>
       <x:c r="J12" s="106"/>
       <x:c r="K12" s="107"/>
+      <x:c r="L12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="112" t="n">
@@ -1235,6 +1279,7 @@
       <x:c r="I13" s="128"/>
       <x:c r="J13" s="68"/>
       <x:c r="K13" s="69"/>
+      <x:c r="L13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="113" t="n">
@@ -1250,6 +1295,7 @@
       <x:c r="I14" s="129"/>
       <x:c r="J14" s="106"/>
       <x:c r="K14" s="107"/>
+      <x:c r="L14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="112" t="n">
@@ -1265,6 +1311,7 @@
       <x:c r="I15" s="128"/>
       <x:c r="J15" s="68"/>
       <x:c r="K15" s="69"/>
+      <x:c r="L15"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="113" t="n">
@@ -1280,6 +1327,7 @@
       <x:c r="I16" s="129"/>
       <x:c r="J16" s="106"/>
       <x:c r="K16" s="107"/>
+      <x:c r="L16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="112" t="n">
@@ -1295,6 +1343,7 @@
       <x:c r="I17" s="128"/>
       <x:c r="J17" s="68"/>
       <x:c r="K17" s="69"/>
+      <x:c r="L17"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="113" t="n">
@@ -1310,6 +1359,7 @@
       <x:c r="I18" s="129"/>
       <x:c r="J18" s="106"/>
       <x:c r="K18" s="107"/>
+      <x:c r="L18"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="112" t="n">
@@ -1325,6 +1375,7 @@
       <x:c r="I19" s="128"/>
       <x:c r="J19" s="68"/>
       <x:c r="K19" s="69"/>
+      <x:c r="L19"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="113" t="n">
@@ -1340,6 +1391,7 @@
       <x:c r="I20" s="129"/>
       <x:c r="J20" s="106"/>
       <x:c r="K20" s="107"/>
+      <x:c r="L20"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="112" t="n">
@@ -1355,6 +1407,7 @@
       <x:c r="I21" s="128"/>
       <x:c r="J21" s="68"/>
       <x:c r="K21" s="69"/>
+      <x:c r="L21"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="113" t="n">
@@ -1370,6 +1423,7 @@
       <x:c r="I22" s="129"/>
       <x:c r="J22" s="106"/>
       <x:c r="K22" s="107"/>
+      <x:c r="L22"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="112" t="n">
@@ -1385,6 +1439,7 @@
       <x:c r="I23" s="128"/>
       <x:c r="J23" s="68"/>
       <x:c r="K23" s="69"/>
+      <x:c r="L23"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="113" t="n">
@@ -1400,6 +1455,7 @@
       <x:c r="I24" s="129"/>
       <x:c r="J24" s="106"/>
       <x:c r="K24" s="107"/>
+      <x:c r="L24"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="112" t="n">
@@ -1415,6 +1471,7 @@
       <x:c r="I25" s="128"/>
       <x:c r="J25" s="68"/>
       <x:c r="K25" s="69"/>
+      <x:c r="L25"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="113" t="n">
@@ -1430,6 +1487,7 @@
       <x:c r="I26" s="129"/>
       <x:c r="J26" s="106"/>
       <x:c r="K26" s="107"/>
+      <x:c r="L26"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="112" t="n">
@@ -1445,6 +1503,7 @@
       <x:c r="I27" s="128"/>
       <x:c r="J27" s="68"/>
       <x:c r="K27" s="69"/>
+      <x:c r="L27"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="113" t="n">
@@ -1460,6 +1519,7 @@
       <x:c r="I28" s="129"/>
       <x:c r="J28" s="106"/>
       <x:c r="K28" s="107"/>
+      <x:c r="L28"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="112" t="n">
@@ -1475,6 +1535,7 @@
       <x:c r="I29" s="128"/>
       <x:c r="J29" s="68"/>
       <x:c r="K29" s="69"/>
+      <x:c r="L29"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="113" t="n">
@@ -1490,6 +1551,7 @@
       <x:c r="I30" s="129"/>
       <x:c r="J30" s="106"/>
       <x:c r="K30" s="107"/>
+      <x:c r="L30"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="112" t="n">
@@ -1505,6 +1567,7 @@
       <x:c r="I31" s="128"/>
       <x:c r="J31" s="68"/>
       <x:c r="K31" s="69"/>
+      <x:c r="L31"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="113" t="n">
@@ -1520,6 +1583,7 @@
       <x:c r="I32" s="129"/>
       <x:c r="J32" s="106"/>
       <x:c r="K32" s="107"/>
+      <x:c r="L32"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="112" t="n">
@@ -1535,6 +1599,7 @@
       <x:c r="I33" s="128"/>
       <x:c r="J33" s="68"/>
       <x:c r="K33" s="69"/>
+      <x:c r="L33"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="113" t="n">
@@ -1550,6 +1615,7 @@
       <x:c r="I34" s="129"/>
       <x:c r="J34" s="106"/>
       <x:c r="K34" s="107"/>
+      <x:c r="L34"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="112" t="n">
@@ -1565,6 +1631,7 @@
       <x:c r="I35" s="128"/>
       <x:c r="J35" s="68"/>
       <x:c r="K35" s="69"/>
+      <x:c r="L35"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="113" t="n">
@@ -1580,6 +1647,7 @@
       <x:c r="I36" s="129"/>
       <x:c r="J36" s="106"/>
       <x:c r="K36" s="107"/>
+      <x:c r="L36"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="112" t="n">
@@ -1595,6 +1663,7 @@
       <x:c r="I37" s="128"/>
       <x:c r="J37" s="68"/>
       <x:c r="K37" s="69"/>
+      <x:c r="L37"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="113" t="n">
@@ -1610,6 +1679,7 @@
       <x:c r="I38" s="129"/>
       <x:c r="J38" s="106"/>
       <x:c r="K38" s="107"/>
+      <x:c r="L38"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="112" t="n">
@@ -1625,6 +1695,7 @@
       <x:c r="I39" s="128"/>
       <x:c r="J39" s="68"/>
       <x:c r="K39" s="69"/>
+      <x:c r="L39"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="113" t="n">
@@ -1640,6 +1711,7 @@
       <x:c r="I40" s="129"/>
       <x:c r="J40" s="106"/>
       <x:c r="K40" s="107"/>
+      <x:c r="L40"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="112" t="n">
@@ -1655,6 +1727,7 @@
       <x:c r="I41" s="128"/>
       <x:c r="J41" s="68"/>
       <x:c r="K41" s="69"/>
+      <x:c r="L41"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="113" t="n">
@@ -1670,6 +1743,7 @@
       <x:c r="I42" s="129"/>
       <x:c r="J42" s="106"/>
       <x:c r="K42" s="107"/>
+      <x:c r="L42"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="112" t="n">
@@ -1685,6 +1759,7 @@
       <x:c r="I43" s="128"/>
       <x:c r="J43" s="68"/>
       <x:c r="K43" s="69"/>
+      <x:c r="L43"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="113" t="n">
@@ -1700,6 +1775,7 @@
       <x:c r="I44" s="129"/>
       <x:c r="J44" s="106"/>
       <x:c r="K44" s="107"/>
+      <x:c r="L44"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="112" t="n">
@@ -1715,6 +1791,7 @@
       <x:c r="I45" s="128"/>
       <x:c r="J45" s="68"/>
       <x:c r="K45" s="69"/>
+      <x:c r="L45"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="113" t="n">
@@ -1730,6 +1807,7 @@
       <x:c r="I46" s="129"/>
       <x:c r="J46" s="106"/>
       <x:c r="K46" s="107"/>
+      <x:c r="L46"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="112" t="n">
@@ -1745,6 +1823,7 @@
       <x:c r="I47" s="128"/>
       <x:c r="J47" s="68"/>
       <x:c r="K47" s="69"/>
+      <x:c r="L47"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="113" t="n">
@@ -1760,6 +1839,7 @@
       <x:c r="I48" s="129"/>
       <x:c r="J48" s="106"/>
       <x:c r="K48" s="107"/>
+      <x:c r="L48"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="112" t="n">
@@ -1775,6 +1855,7 @@
       <x:c r="I49" s="128"/>
       <x:c r="J49" s="68"/>
       <x:c r="K49" s="69"/>
+      <x:c r="L49"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="113" t="n">
@@ -1790,6 +1871,7 @@
       <x:c r="I50" s="129"/>
       <x:c r="J50" s="106"/>
       <x:c r="K50" s="107"/>
+      <x:c r="L50"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="112" t="n">
@@ -1805,6 +1887,7 @@
       <x:c r="I51" s="128"/>
       <x:c r="J51" s="68"/>
       <x:c r="K51" s="69"/>
+      <x:c r="L51"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="113" t="n">
@@ -1820,6 +1903,7 @@
       <x:c r="I52" s="129"/>
       <x:c r="J52" s="106"/>
       <x:c r="K52" s="107"/>
+      <x:c r="L52"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="114" t="n">
@@ -1835,17 +1919,18 @@
       <x:c r="I53" s="130"/>
       <x:c r="J53" s="71"/>
       <x:c r="K53" s="72"/>
+      <x:c r="L53"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:K1"/>
-    <x:mergeCell ref="A2:K2"/>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="G4:G53">
+    <x:dataValidation type="list" sqref="H4:H53">
       <x:formula1>"Nam,Nữ,Khác"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K4:K53">
+    <x:dataValidation type="list" sqref="L4:L53">
       <x:formula1>"Đang học,Tạm nghỉ,Đã tốt nghiệp"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -1868,6 +1953,7 @@
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1875,7 +1961,7 @@
         <x:v>MẪU NHẬP SINH VIÊN THEO LỚP HÀNH CHÍNH - VÍ DỤ</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="151" t="str">
         <x:v>STT</x:v>
       </x:c>
@@ -1892,21 +1978,24 @@
         <x:v>Mật khẩu</x:v>
       </x:c>
       <x:c r="F3" s="152" t="str">
+        <x:v>Mã lớp</x:v>
+      </x:c>
+      <x:c r="G3" s="152" t="str">
         <x:v>Ngày sinh</x:v>
       </x:c>
-      <x:c r="G3" s="152" t="str">
+      <x:c r="H3" s="152" t="str">
         <x:v>Giới tính</x:v>
       </x:c>
-      <x:c r="H3" s="152" t="str">
+      <x:c r="I3" s="152" t="str">
         <x:v>Số điện thoại</x:v>
       </x:c>
-      <x:c r="I3" s="152" t="str">
+      <x:c r="J3" s="152" t="str">
         <x:v>CCCD</x:v>
       </x:c>
-      <x:c r="J3" s="152" t="str">
+      <x:c r="K3" s="153" t="str">
         <x:v>Địa chỉ</x:v>
       </x:c>
-      <x:c r="K3" s="153" t="str">
+      <x:c r="L3" s="235" t="str">
         <x:v>Trạng thái sinh viên</x:v>
       </x:c>
     </x:row>
@@ -1927,28 +2016,39 @@
         <x:v>123456</x:v>
       </x:c>
       <x:c r="F4" s="170" t="str">
+        <x:v>CNTT2601</x:v>
+      </x:c>
+      <x:c r="G4" s="170" t="str">
         <x:v>02/02/2006</x:v>
       </x:c>
-      <x:c r="G4" s="170" t="str">
+      <x:c r="H4" s="170" t="str">
         <x:v>Nữ</x:v>
       </x:c>
-      <x:c r="H4" s="170" t="str">
+      <x:c r="I4" s="170" t="str">
         <x:v>0900000002</x:v>
       </x:c>
-      <x:c r="I4" s="170" t="str">
+      <x:c r="J4" s="170" t="str">
         <x:v>012345678902</x:v>
       </x:c>
-      <x:c r="J4" s="170" t="str">
+      <x:c r="K4" s="171" t="str">
         <x:v>Cần Thơ</x:v>
       </x:c>
-      <x:c r="K4" s="171" t="str">
+      <x:c r="L4" t="str">
         <x:v>Đang học</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:K1"/>
+    <x:mergeCell ref="A1:L1"/>
   </x:mergeCells>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="H4">
+      <x:formula1>"Nam,Nữ,Khác"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="L4">
+      <x:formula1>"Đang học,Tạm nghỉ,Đã tốt nghiệp"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -2003,7 +2103,7 @@
         <x:v>Cột bắt buộc</x:v>
       </x:c>
       <x:c r="B7" s="200" t="str">
-        <x:v>Mã sinh viên, Họ tên, Email, Mật khẩu</x:v>
+        <x:v>Mã sinh viên, Họ tên, Email, Mật khẩu, Mã lớp</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2011,7 +2111,7 @@
         <x:v>Lớp hành chính</x:v>
       </x:c>
       <x:c r="B8" s="200" t="str">
-        <x:v>Phải chọn Mã lớp hành chính đích trên màn hình Nhập Excel trước khi kiểm tra.</x:v>
+        <x:v>Nhập Mã lớp ngay trên từng dòng sinh viên. Có thể nhập sinh viên của nhiều lớp trong cùng một file.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2019,7 +2119,7 @@
         <x:v>Tự động liên kết</x:v>
       </x:c>
       <x:c r="B9" s="200" t="str">
-        <x:v>Hệ thống tự lấy Lớp, Mã khoa và Khóa học từ lớp đã chọn.</x:v>
+        <x:v>Hệ thống tìm lớp trùng Mã lớp, sau đó tự lấy Khoa và Khóa học từ năm nhập học của lớp.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">

</xml_diff>